<commit_message>
feat: improve planner item workflows and automate PNG icon registration
Preserve function drafts, clarify Excel exports, improve readability, and update validation contracts. Add portable PNG icon bundles and Unity Sprite/Addressables importer. Use BACKND persistent chart updates and log unchanged data reuse.
</commit_message>
<xml_diff>
--- a/tools/planner-studio/app/seeds/UnitBalance.xlsx
+++ b/tools/planner-studio/app/seeds/UnitBalance.xlsx
@@ -430,7 +430,7 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -457,7 +457,7 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -484,7 +484,7 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G5">
         <v>0</v>

</xml_diff>